<commit_message>
Commit 3: Actualización de la Carpeta 3 con base de datos, scripts y documentación
</commit_message>
<xml_diff>
--- a/Carpeta_N3_Base_de_datos_y_codigo/salidas/tabla1_estadisticas_descriptivas.xlsx
+++ b/Carpeta_N3_Base_de_datos_y_codigo/salidas/tabla1_estadisticas_descriptivas.xlsx
@@ -413,82 +413,82 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>grupo</t>
+          <t>variable</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>n</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>mean</t>
+          <t>media</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>std</t>
+          <t>desv_estandar</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>min</t>
+          <t>minimo</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>p25</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>mediana</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>75%</t>
+          <t>p75</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>max</t>
+          <t>maximo</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Todo el panel</t>
+          <t>Ratio de Capital Global (%)</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2112</v>
+        <v>1920</v>
       </c>
       <c r="C2" t="n">
-        <v>27.51</v>
+        <v>28.78</v>
       </c>
       <c r="D2" t="n">
-        <v>64.48999999999999</v>
+        <v>67.51000000000001</v>
       </c>
       <c r="E2" t="n">
         <v>4.22</v>
       </c>
       <c r="F2" t="n">
-        <v>14</v>
+        <v>14.11</v>
       </c>
       <c r="G2" t="n">
         <v>15.51</v>
       </c>
       <c r="H2" t="n">
-        <v>17.92</v>
+        <v>18.77</v>
       </c>
       <c r="I2" t="n">
         <v>513.77</v>
@@ -497,63 +497,94 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SBS_original</t>
+          <t>ROE anualizado (%)</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1419</v>
+        <v>1920</v>
       </c>
       <c r="C3" t="n">
-        <v>21.73</v>
+        <v>-55.69</v>
       </c>
       <c r="D3" t="n">
-        <v>29.31</v>
+        <v>274.73</v>
       </c>
       <c r="E3" t="n">
-        <v>4.22</v>
+        <v>-1605.51</v>
       </c>
       <c r="F3" t="n">
-        <v>14.22</v>
+        <v>1.31</v>
       </c>
       <c r="G3" t="n">
-        <v>15.59</v>
+        <v>8.279999999999999</v>
       </c>
       <c r="H3" t="n">
-        <v>18.87</v>
+        <v>15.34</v>
       </c>
       <c r="I3" t="n">
-        <v>513.77</v>
+        <v>44.21</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>interpolado</t>
+          <t>Cartera Atrasada (%)</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>693</v>
+        <v>1920</v>
       </c>
       <c r="C4" t="n">
-        <v>39.34</v>
+        <v>3.56</v>
       </c>
       <c r="D4" t="n">
-        <v>103.53</v>
+        <v>2.62</v>
       </c>
       <c r="E4" t="n">
-        <v>4.52</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>12.3</v>
+        <v>2.48</v>
       </c>
       <c r="G4" t="n">
-        <v>14.89</v>
+        <v>3.37</v>
       </c>
       <c r="H4" t="n">
-        <v>16.99</v>
+        <v>4.75</v>
       </c>
       <c r="I4" t="n">
-        <v>513.77</v>
+        <v>22.7</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>APR total (miles de S/.)</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1920</v>
+      </c>
+      <c r="C5" t="n">
+        <v>24738925.91</v>
+      </c>
+      <c r="D5" t="n">
+        <v>38491393.27</v>
+      </c>
+      <c r="E5" t="n">
+        <v>50586.7</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1458963.06</v>
+      </c>
+      <c r="G5" t="n">
+        <v>5047462.97</v>
+      </c>
+      <c r="H5" t="n">
+        <v>23909151.47</v>
+      </c>
+      <c r="I5" t="n">
+        <v>170718149.25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>